<commit_message>
Update workbook with labor hours check
</commit_message>
<xml_diff>
--- a/capabilities/marginal-analysis/model.xlsx
+++ b/capabilities/marginal-analysis/model.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/talaivosamoala/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91AA7A67-AF07-F94E-8633-14E24DC4C09B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60AB3F35-AFBB-CA4D-82FE-8103FB0E6EB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="17180" yWindow="940" windowWidth="16880" windowHeight="19340" firstSheet="3" activeTab="8" xr2:uid="{C0270FAA-BF4C-9A43-9A85-05328FDD9A3B}"/>
+    <workbookView xWindow="15800" yWindow="980" windowWidth="16880" windowHeight="19340" firstSheet="3" activeTab="5" xr2:uid="{C0270FAA-BF4C-9A43-9A85-05328FDD9A3B}"/>
   </bookViews>
   <sheets>
     <sheet name="Inputs" sheetId="1" r:id="rId1"/>
@@ -70,7 +70,7 @@
     <definedName name="solver_val" localSheetId="9" hidden="1">0</definedName>
     <definedName name="solver_ver" localSheetId="9" hidden="1">2</definedName>
   </definedNames>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -94,7 +94,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="115">
   <si>
     <t>Named_Range</t>
   </si>
@@ -436,6 +436,9 @@
   </si>
   <si>
     <t xml:space="preserve">Total_Profit </t>
+  </si>
+  <si>
+    <t>Labor_Hours_Check</t>
   </si>
 </sst>
 </file>
@@ -446,7 +449,7 @@
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
     <numFmt numFmtId="166" formatCode="0.0000"/>
-    <numFmt numFmtId="169" formatCode="0.0000000"/>
+    <numFmt numFmtId="167" formatCode="0.0000000"/>
   </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -498,7 +501,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1467,7 +1470,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D79AB11-DB20-104E-BD5A-7DA0161C0FD6}">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18.5" bestFit="1" customWidth="1"/>
@@ -1544,6 +1547,15 @@
       </c>
       <c r="C6" t="s">
         <v>62</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>114</v>
+      </c>
+      <c r="B7" t="b">
+        <f>Optimization!B8&lt;=6480</f>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update marginal costs and fixed cost calculation
</commit_message>
<xml_diff>
--- a/capabilities/marginal-analysis/model.xlsx
+++ b/capabilities/marginal-analysis/model.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/talaivosamoala/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60AB3F35-AFBB-CA4D-82FE-8103FB0E6EB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15AE96D9-0BD2-4F41-A763-E66173CB1049}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15800" yWindow="980" windowWidth="16880" windowHeight="19340" firstSheet="3" activeTab="5" xr2:uid="{C0270FAA-BF4C-9A43-9A85-05328FDD9A3B}"/>
+    <workbookView xWindow="17180" yWindow="940" windowWidth="16880" windowHeight="19360" firstSheet="3" activeTab="9" xr2:uid="{C0270FAA-BF4C-9A43-9A85-05328FDD9A3B}"/>
   </bookViews>
   <sheets>
     <sheet name="Inputs" sheetId="1" r:id="rId1"/>
@@ -94,7 +94,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="121">
   <si>
     <t>Named_Range</t>
   </si>
@@ -439,6 +439,24 @@
   </si>
   <si>
     <t>Labor_Hours_Check</t>
+  </si>
+  <si>
+    <t>Tomato_Marginal_Cost</t>
+  </si>
+  <si>
+    <t>Carrot_Marginal_Cost</t>
+  </si>
+  <si>
+    <t>Carrot_Added_Labor_Dollars</t>
+  </si>
+  <si>
+    <t>Mesclun_Marginal_Cost</t>
+  </si>
+  <si>
+    <t>Mesclun_Added_Labor_Dollars</t>
+  </si>
+  <si>
+    <t>Season_Fixed_Costs</t>
   </si>
 </sst>
 </file>
@@ -451,13 +469,19 @@
     <numFmt numFmtId="166" formatCode="0.0000"/>
     <numFmt numFmtId="167" formatCode="0.0000000"/>
   </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -480,7 +504,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -502,6 +526,7 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -836,7 +861,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B3232F0-D3C9-8A4B-8877-5023CEFADCDF}">
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="24" bestFit="1" customWidth="1"/>
@@ -1062,6 +1087,14 @@
       </c>
       <c r="C20" s="1" t="s">
         <v>24</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A21" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="B21" s="1">
+        <v>20000</v>
       </c>
     </row>
   </sheetData>
@@ -1178,8 +1211,8 @@
         <v>113</v>
       </c>
       <c r="B13">
-        <f>B10-B11-B12</f>
-        <v>62775.155387742139</v>
+        <f>B10-B11-B12-Inputs!B21</f>
+        <v>42775.155387742139</v>
       </c>
     </row>
   </sheetData>
@@ -1689,7 +1722,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AF2FFFE8-48B8-384E-AFF2-E7D9BD69847B}">
-  <dimension ref="A1:AB31"/>
+  <dimension ref="A1:AG31"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.6640625" bestFit="1" customWidth="1"/>
@@ -1714,9 +1747,14 @@
     <col min="26" max="26" width="24.83203125" bestFit="1" customWidth="1"/>
     <col min="27" max="27" width="25.6640625" bestFit="1" customWidth="1"/>
     <col min="28" max="28" width="26.33203125" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="19.83203125" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="19.1640625" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="24.6640625" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="20.6640625" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="26.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:33" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1777,8 +1815,23 @@
       <c r="AB1" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC1" t="s">
+        <v>115</v>
+      </c>
+      <c r="AD1" t="s">
+        <v>116</v>
+      </c>
+      <c r="AE1" t="s">
+        <v>117</v>
+      </c>
+      <c r="AF1" t="s">
+        <v>118</v>
+      </c>
+      <c r="AG1" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="2" spans="1:33" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>76</v>
       </c>
@@ -1878,8 +1931,28 @@
         <f>Z2*Inputs!B20</f>
         <v>150401.62366512578</v>
       </c>
-    </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC2">
+        <f>H2+I2</f>
+        <v>4317.2800000000007</v>
+      </c>
+      <c r="AD2">
+        <f>AE2+R2</f>
+        <v>1507.2129439999999</v>
+      </c>
+      <c r="AE2">
+        <f>M2*Inputs!$B$19</f>
+        <v>1067.2129439999999</v>
+      </c>
+      <c r="AF2">
+        <f>AG2+S2</f>
+        <v>2461.9299999999998</v>
+      </c>
+      <c r="AG2">
+        <f>Q2*Inputs!$B$19</f>
+        <v>1581.9299999999998</v>
+      </c>
+    </row>
+    <row r="3" spans="1:33" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>78</v>
       </c>
@@ -1939,8 +2012,28 @@
         <f>Inputs!$B$13</f>
         <v>880</v>
       </c>
-    </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC3">
+        <f t="shared" ref="AC3:AC21" si="0">H3+I3</f>
+        <v>5004.7360000000008</v>
+      </c>
+      <c r="AD3">
+        <f t="shared" ref="AD3:AD21" si="1">AE3+R3</f>
+        <v>1560.5735911999998</v>
+      </c>
+      <c r="AE3">
+        <f>M3*Inputs!$B$19</f>
+        <v>1120.5735911999998</v>
+      </c>
+      <c r="AF3">
+        <f t="shared" ref="AF3:AF31" si="2">AG3+S3</f>
+        <v>2501.4782499999997</v>
+      </c>
+      <c r="AG3">
+        <f>Q3*Inputs!$B$19</f>
+        <v>1621.4782499999997</v>
+      </c>
+    </row>
+    <row r="4" spans="1:33" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>80</v>
       </c>
@@ -1959,7 +2052,7 @@
         <v>359.37000000000012</v>
       </c>
       <c r="G4">
-        <f t="shared" ref="G4:G21" si="0">F4-F3</f>
+        <f t="shared" ref="G4:G21" si="3">F4-F3</f>
         <v>141.57000000000008</v>
       </c>
       <c r="H4">
@@ -1978,7 +2071,7 @@
         <v>96.881388187499979</v>
       </c>
       <c r="M4">
-        <f t="shared" ref="M4:M21" si="1">L4-L3</f>
+        <f t="shared" ref="M4:M21" si="4">L4-L3</f>
         <v>33.869103187499988</v>
       </c>
       <c r="O4">
@@ -1989,7 +2082,7 @@
         <v>140.12604492187498</v>
       </c>
       <c r="Q4">
-        <f t="shared" ref="Q4:Q31" si="2">P4-P3</f>
+        <f t="shared" ref="Q4:Q31" si="5">P4-P3</f>
         <v>47.861982421874984</v>
       </c>
       <c r="R4">
@@ -2000,8 +2093,28 @@
         <f>Inputs!$B$13</f>
         <v>880</v>
       </c>
-    </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC4">
+        <f t="shared" si="0"/>
+        <v>5795.3104000000021</v>
+      </c>
+      <c r="AD4">
+        <f t="shared" si="1"/>
+        <v>1615.9352626699995</v>
+      </c>
+      <c r="AE4">
+        <f>M4*Inputs!$B$19</f>
+        <v>1175.9352626699995</v>
+      </c>
+      <c r="AF4">
+        <f t="shared" si="2"/>
+        <v>2541.7680296874996</v>
+      </c>
+      <c r="AG4">
+        <f>Q4*Inputs!$B$19</f>
+        <v>1661.7680296874994</v>
+      </c>
+    </row>
+    <row r="5" spans="1:33" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>82</v>
       </c>
@@ -2020,7 +2133,7 @@
         <v>527.07600000000014</v>
       </c>
       <c r="G5">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>167.70600000000002</v>
       </c>
       <c r="H5">
@@ -2039,7 +2152,7 @@
         <v>132.40456385624998</v>
       </c>
       <c r="M5">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>35.52317566875</v>
       </c>
       <c r="O5">
@@ -2050,7 +2163,7 @@
         <v>189.17016064453125</v>
       </c>
       <c r="Q5">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>49.044115722656272</v>
       </c>
       <c r="R5">
@@ -2061,8 +2174,28 @@
         <f>Inputs!$B$13</f>
         <v>880</v>
       </c>
-    </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC5">
+        <f t="shared" si="0"/>
+        <v>6702.7523200000005</v>
+      </c>
+      <c r="AD5">
+        <f t="shared" si="1"/>
+        <v>1673.364659219</v>
+      </c>
+      <c r="AE5">
+        <f>M5*Inputs!$B$19</f>
+        <v>1233.364659219</v>
+      </c>
+      <c r="AF5">
+        <f t="shared" si="2"/>
+        <v>2582.8116978906255</v>
+      </c>
+      <c r="AG5">
+        <f>Q5*Inputs!$B$19</f>
+        <v>1702.8116978906257</v>
+      </c>
+    </row>
+    <row r="6" spans="1:33" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>84</v>
       </c>
@@ -2081,7 +2214,7 @@
         <v>724.72950000000026</v>
       </c>
       <c r="G6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>197.65350000000012</v>
       </c>
       <c r="H6">
@@ -2100,7 +2233,7 @@
         <v>169.64334744082026</v>
       </c>
       <c r="M6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>37.238783584570285</v>
       </c>
       <c r="O6">
@@ -2111,7 +2244,7 @@
         <v>239.41848456573481</v>
       </c>
       <c r="Q6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>50.248323921203564</v>
       </c>
       <c r="R6">
@@ -2122,8 +2255,28 @@
         <f>Inputs!$B$13</f>
         <v>880</v>
       </c>
-    </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC6">
+        <f t="shared" si="0"/>
+        <v>7660.4253999999992</v>
+      </c>
+      <c r="AD6">
+        <f t="shared" si="1"/>
+        <v>1732.9305660562802</v>
+      </c>
+      <c r="AE6">
+        <f>M6*Inputs!$B$19</f>
+        <v>1292.9305660562802</v>
+      </c>
+      <c r="AF6">
+        <f t="shared" si="2"/>
+        <v>2624.6218065441876</v>
+      </c>
+      <c r="AG6">
+        <f>Q6*Inputs!$B$19</f>
+        <v>1744.6218065441876</v>
+      </c>
+    </row>
+    <row r="7" spans="1:33" x14ac:dyDescent="0.2">
       <c r="E7" s="9">
         <v>6</v>
       </c>
@@ -2132,7 +2285,7 @@
         <v>956.64294000000041</v>
       </c>
       <c r="G7">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>231.91344000000015</v>
       </c>
       <c r="H7">
@@ -2151,7 +2304,7 @@
         <v>208.66131735220887</v>
       </c>
       <c r="M7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>39.017969911388604</v>
       </c>
       <c r="O7">
@@ -2162,7 +2315,7 @@
         <v>290.89345874736784</v>
       </c>
       <c r="Q7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>51.47497418163303</v>
       </c>
       <c r="R7">
@@ -2173,8 +2326,28 @@
         <f>Inputs!$B$13</f>
         <v>880</v>
       </c>
-    </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC7">
+        <f t="shared" si="0"/>
+        <v>4906.0173184000023</v>
+      </c>
+      <c r="AD7">
+        <f t="shared" si="1"/>
+        <v>1794.7039153234123</v>
+      </c>
+      <c r="AE7">
+        <f>M7*Inputs!$B$19</f>
+        <v>1354.7039153234123</v>
+      </c>
+      <c r="AF7">
+        <f t="shared" si="2"/>
+        <v>2667.211103586299</v>
+      </c>
+      <c r="AG7">
+        <f>Q7*Inputs!$B$19</f>
+        <v>1787.2111035862988</v>
+      </c>
+    </row>
+    <row r="8" spans="1:33" x14ac:dyDescent="0.2">
       <c r="E8" s="9">
         <v>7</v>
       </c>
@@ -2183,7 +2356,7 @@
         <v>1227.6917730000007</v>
       </c>
       <c r="G8">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>271.04883300000029</v>
       </c>
       <c r="H8">
@@ -2202,7 +2375,7 @@
         <v>249.52415866701648</v>
       </c>
       <c r="M8">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>40.862841314807611</v>
       </c>
       <c r="O8">
@@ -2213,7 +2386,7 @@
         <v>343.61789814532818</v>
       </c>
       <c r="Q8">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>52.724439397960339</v>
       </c>
       <c r="R8">
@@ -2224,8 +2397,28 @@
         <f>Inputs!$B$13</f>
         <v>880</v>
       </c>
-    </row>
-    <row r="9" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC8">
+        <f t="shared" si="0"/>
+        <v>5585.4077408800049</v>
+      </c>
+      <c r="AD8">
+        <f t="shared" si="1"/>
+        <v>1858.7578504501203</v>
+      </c>
+      <c r="AE8">
+        <f>M8*Inputs!$B$19</f>
+        <v>1418.7578504501203</v>
+      </c>
+      <c r="AF8">
+        <f t="shared" si="2"/>
+        <v>2710.5925358971826</v>
+      </c>
+      <c r="AG8">
+        <f>Q8*Inputs!$B$19</f>
+        <v>1830.5925358971829</v>
+      </c>
+    </row>
+    <row r="9" spans="1:33" x14ac:dyDescent="0.2">
       <c r="E9" s="9">
         <v>8</v>
       </c>
@@ -2234,7 +2427,7 @@
         <v>1543.3839432000009</v>
       </c>
       <c r="G9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>315.69217020000019</v>
       </c>
       <c r="H9">
@@ -2253,7 +2446,7 @@
         <v>292.29972872421928</v>
       </c>
       <c r="M9">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>42.775570057202799</v>
       </c>
       <c r="O9">
@@ -2264,7 +2457,7 @@
         <v>397.61499642530839</v>
       </c>
       <c r="Q9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>53.997098279980207</v>
       </c>
       <c r="R9">
@@ -2275,8 +2468,28 @@
         <f>Inputs!$B$13</f>
         <v>880</v>
       </c>
-    </row>
-    <row r="10" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC9">
+        <f t="shared" si="0"/>
+        <v>6360.4160746720036</v>
+      </c>
+      <c r="AD9">
+        <f t="shared" si="1"/>
+        <v>1925.1677923860811</v>
+      </c>
+      <c r="AE9">
+        <f>M9*Inputs!$B$19</f>
+        <v>1485.1677923860811</v>
+      </c>
+      <c r="AF9">
+        <f t="shared" si="2"/>
+        <v>2754.7792522809127</v>
+      </c>
+      <c r="AG9">
+        <f>Q9*Inputs!$B$19</f>
+        <v>1874.7792522809127</v>
+      </c>
+    </row>
+    <row r="10" spans="1:33" x14ac:dyDescent="0.2">
       <c r="E10" s="9">
         <v>9</v>
       </c>
@@ -2285,7 +2498,7 @@
         <v>1909.9376297100011</v>
       </c>
       <c r="G10">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>366.55368651000026</v>
       </c>
       <c r="H10">
@@ -2304,7 +2517,7 @@
         <v>337.05812468511533</v>
       </c>
       <c r="M10">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>44.758395960896053</v>
       </c>
       <c r="O10">
@@ -2315,7 +2528,7 @@
         <v>452.90833186570285</v>
       </c>
       <c r="Q10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>55.293335440394458</v>
       </c>
       <c r="R10">
@@ -2326,8 +2539,28 @@
         <f>Inputs!$B$13</f>
         <v>880</v>
       </c>
-    </row>
-    <row r="11" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC10">
+        <f t="shared" si="0"/>
+        <v>7243.3719978136041</v>
+      </c>
+      <c r="AD10">
+        <f t="shared" si="1"/>
+        <v>1994.0115077623109</v>
+      </c>
+      <c r="AE10">
+        <f>M10*Inputs!$B$19</f>
+        <v>1554.0115077623109</v>
+      </c>
+      <c r="AF10">
+        <f t="shared" si="2"/>
+        <v>2799.7846064904952</v>
+      </c>
+      <c r="AG10">
+        <f>Q10*Inputs!$B$19</f>
+        <v>1919.7846064904954</v>
+      </c>
+    </row>
+    <row r="11" spans="1:33" x14ac:dyDescent="0.2">
       <c r="E11" s="9">
         <v>10</v>
       </c>
@@ -2336,7 +2569,7 @@
         <v>2334.3682140900019</v>
       </c>
       <c r="G11">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>424.43058438000071</v>
       </c>
       <c r="H11">
@@ -2355,7 +2588,7 @@
         <v>383.87175311360357</v>
       </c>
       <c r="M11">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>46.813628428488244</v>
       </c>
       <c r="O11">
@@ -2366,7 +2599,7 @@
         <v>509.52187334891573</v>
       </c>
       <c r="Q11">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>56.613541483212884</v>
       </c>
       <c r="R11">
@@ -2377,8 +2610,28 @@
         <f>Inputs!$B$13</f>
         <v>880</v>
       </c>
-    </row>
-    <row r="12" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC11">
+        <f t="shared" si="0"/>
+        <v>8248.1149448368124</v>
+      </c>
+      <c r="AD11">
+        <f t="shared" si="1"/>
+        <v>2065.3691790371117</v>
+      </c>
+      <c r="AE11">
+        <f>M11*Inputs!$B$19</f>
+        <v>1625.3691790371117</v>
+      </c>
+      <c r="AF11">
+        <f t="shared" si="2"/>
+        <v>2845.6221602971514</v>
+      </c>
+      <c r="AG11">
+        <f>Q11*Inputs!$B$19</f>
+        <v>1965.6221602971514</v>
+      </c>
+    </row>
+    <row r="12" spans="1:33" x14ac:dyDescent="0.2">
       <c r="E12" s="9">
         <v>11</v>
       </c>
@@ -2387,7 +2640,7 @@
         <v>2824.5855390489023</v>
       </c>
       <c r="G12">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>490.21732495890046</v>
       </c>
       <c r="H12">
@@ -2406,7 +2659,7 @@
         <v>432.81540163558799</v>
       </c>
       <c r="M12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>48.943648521984414</v>
       </c>
       <c r="O12">
@@ -2417,7 +2670,7 @@
         <v>567.47998644235474</v>
       </c>
       <c r="Q12">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>57.95811309343901</v>
       </c>
       <c r="R12">
@@ -2428,8 +2681,28 @@
         <f>Inputs!$B$13</f>
         <v>880</v>
       </c>
-    </row>
-    <row r="13" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC12">
+        <f t="shared" si="0"/>
+        <v>9390.1727612865125</v>
+      </c>
+      <c r="AD12">
+        <f t="shared" si="1"/>
+        <v>2139.3234766832988</v>
+      </c>
+      <c r="AE12">
+        <f>M12*Inputs!$B$19</f>
+        <v>1699.3234766832988</v>
+      </c>
+      <c r="AF12">
+        <f t="shared" si="2"/>
+        <v>2892.3056866042025</v>
+      </c>
+      <c r="AG12">
+        <f>Q12*Inputs!$B$19</f>
+        <v>2012.3056866042023</v>
+      </c>
+    </row>
+    <row r="13" spans="1:33" x14ac:dyDescent="0.2">
       <c r="E13" s="9">
         <v>12</v>
       </c>
@@ -2438,7 +2711,7 @@
         <v>3389.502646858683</v>
       </c>
       <c r="G13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>564.91710780978065</v>
       </c>
       <c r="H13">
@@ -2457,7 +2730,7 @@
         <v>483.96631273797556</v>
       </c>
       <c r="M13">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>51.150911102387568</v>
       </c>
       <c r="O13">
@@ -2468,7 +2741,7 @@
         <v>626.80743957041921</v>
       </c>
       <c r="Q13">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>59.327453128064462</v>
       </c>
       <c r="R13">
@@ -2479,8 +2752,28 @@
         <f>Inputs!$B$13</f>
         <v>880</v>
       </c>
-    </row>
-    <row r="14" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC13">
+        <f t="shared" si="0"/>
+        <v>10686.960991577791</v>
+      </c>
+      <c r="AD13">
+        <f t="shared" si="1"/>
+        <v>2215.9596334748962</v>
+      </c>
+      <c r="AE13">
+        <f>M13*Inputs!$B$19</f>
+        <v>1775.9596334748962</v>
+      </c>
+      <c r="AF13">
+        <f t="shared" si="2"/>
+        <v>2939.849172606398</v>
+      </c>
+      <c r="AG13">
+        <f>Q13*Inputs!$B$19</f>
+        <v>2059.849172606398</v>
+      </c>
+    </row>
+    <row r="14" spans="1:33" ht="17" x14ac:dyDescent="0.25">
       <c r="E14" s="9">
         <v>13</v>
       </c>
@@ -2489,7 +2782,7 @@
         <v>4039.1573208399304</v>
       </c>
       <c r="G14">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>649.65467398124747</v>
       </c>
       <c r="H14">
@@ -2508,7 +2801,7 @@
         <v>537.4042597694604</v>
       </c>
       <c r="M14">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>53.437947031484839</v>
       </c>
       <c r="O14">
@@ -2519,7 +2812,7 @@
         <v>687.52941027880343</v>
       </c>
       <c r="Q14">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>60.72197070838422</v>
       </c>
       <c r="R14">
@@ -2530,8 +2823,28 @@
         <f>Inputs!$B$13</f>
         <v>880</v>
       </c>
-    </row>
-    <row r="15" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC14">
+        <f t="shared" si="0"/>
+        <v>12158.005140314455</v>
+      </c>
+      <c r="AD14">
+        <f t="shared" si="1"/>
+        <v>2295.3655209331537</v>
+      </c>
+      <c r="AE14">
+        <f>M14*Inputs!$B$19</f>
+        <v>1855.3655209331534</v>
+      </c>
+      <c r="AF14">
+        <f t="shared" si="2"/>
+        <v>3551.9562605550727</v>
+      </c>
+      <c r="AG14" s="11">
+        <f>(720-P13)*Inputs!$B$19+(P14-720)*Inputs!$B$20</f>
+        <v>2671.9562605550727</v>
+      </c>
+    </row>
+    <row r="15" spans="1:33" x14ac:dyDescent="0.2">
       <c r="E15" s="9">
         <v>14</v>
       </c>
@@ -2540,7 +2853,7 @@
         <v>4784.8479031488414</v>
       </c>
       <c r="G15">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>745.69058230891096</v>
       </c>
       <c r="H15">
@@ -2559,7 +2872,7 @@
         <v>593.2116252070582</v>
       </c>
       <c r="M15">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>55.807365437597809</v>
       </c>
       <c r="O15">
@@ -2570,7 +2883,7 @@
         <v>749.67149159246469</v>
       </c>
       <c r="Q15">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>62.142081313661265</v>
       </c>
       <c r="R15">
@@ -2581,8 +2894,28 @@
         <f>Inputs!$B$13</f>
         <v>880</v>
       </c>
-    </row>
-    <row r="16" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="AC15">
+        <f t="shared" si="0"/>
+        <v>13825.188508882693</v>
+      </c>
+      <c r="AD15">
+        <f t="shared" si="1"/>
+        <v>2377.6317279933955</v>
+      </c>
+      <c r="AE15">
+        <f>M15*Inputs!$B$19</f>
+        <v>1937.6317279933958</v>
+      </c>
+      <c r="AF15">
+        <f t="shared" si="2"/>
+        <v>1958.7865316051596</v>
+      </c>
+      <c r="AG15">
+        <f>Q15*Inputs!$B$20</f>
+        <v>1078.7865316051596</v>
+      </c>
+    </row>
+    <row r="16" spans="1:33" x14ac:dyDescent="0.2">
       <c r="E16" s="9">
         <v>15</v>
       </c>
@@ -2591,7 +2924,7 @@
         <v>5639.2850287111351</v>
       </c>
       <c r="G16">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>854.43712556229366</v>
       </c>
       <c r="H16">
@@ -2610,7 +2943,7 @@
         <v>651.47348125418</v>
       </c>
       <c r="M16">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>58.261856047121796</v>
       </c>
       <c r="O16">
@@ -2621,7 +2954,7 @@
         <v>813.25969846861108</v>
       </c>
       <c r="Q16">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>63.588206876146387</v>
       </c>
       <c r="R16">
@@ -2632,8 +2965,28 @@
         <f>Inputs!$B$13</f>
         <v>880</v>
       </c>
-    </row>
-    <row r="17" spans="5:19" x14ac:dyDescent="0.2">
+      <c r="AC16">
+        <f t="shared" si="0"/>
+        <v>15713.028499761418</v>
+      </c>
+      <c r="AD16">
+        <f t="shared" si="1"/>
+        <v>2462.8516419560688</v>
+      </c>
+      <c r="AE16">
+        <f>M16*Inputs!$B$19</f>
+        <v>2022.8516419560688</v>
+      </c>
+      <c r="AF16">
+        <f t="shared" si="2"/>
+        <v>1983.8912713699012</v>
+      </c>
+      <c r="AG16">
+        <f>Q16*Inputs!$B$20</f>
+        <v>1103.8912713699012</v>
+      </c>
+    </row>
+    <row r="17" spans="5:33" x14ac:dyDescent="0.2">
       <c r="E17" s="9">
         <v>16</v>
       </c>
@@ -2642,7 +2995,7 @@
         <v>6616.761100354398</v>
       </c>
       <c r="G17">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>977.47607164326291</v>
       </c>
       <c r="H17">
@@ -2661,7 +3014,7 @@
         <v>712.27767283790342</v>
       </c>
       <c r="M17">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>60.804191583723423</v>
       </c>
       <c r="O17">
@@ -2672,7 +3025,7 @@
         <v>878.32047434610013</v>
       </c>
       <c r="Q17">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>65.06077587748905</v>
       </c>
       <c r="R17">
@@ -2683,8 +3036,28 @@
         <f>Inputs!$B$13</f>
         <v>880</v>
       </c>
-    </row>
-    <row r="18" spans="5:19" x14ac:dyDescent="0.2">
+      <c r="AC17">
+        <f t="shared" si="0"/>
+        <v>17848.984603727044</v>
+      </c>
+      <c r="AD17">
+        <f t="shared" si="1"/>
+        <v>2551.1215317868773</v>
+      </c>
+      <c r="AE17">
+        <f>M17*Inputs!$B$19</f>
+        <v>2111.1215317868773</v>
+      </c>
+      <c r="AF17">
+        <f t="shared" si="2"/>
+        <v>2009.4550692332098</v>
+      </c>
+      <c r="AG17">
+        <f>Q17*Inputs!$B$20</f>
+        <v>1129.4550692332098</v>
+      </c>
+    </row>
+    <row r="18" spans="5:33" x14ac:dyDescent="0.2">
       <c r="E18" s="9">
         <v>17</v>
       </c>
@@ -2693,7 +3066,7 @@
         <v>7733.3395360392033</v>
       </c>
       <c r="G18">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>1116.5784356848053</v>
       </c>
       <c r="H18">
@@ -2712,7 +3085,7 @@
         <v>775.71490307502916</v>
       </c>
       <c r="M18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>63.437230237125732</v>
       </c>
       <c r="O18">
@@ -2723,7 +3096,7 @@
         <v>944.88069779264049</v>
       </c>
       <c r="Q18">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>66.560223446540363</v>
       </c>
       <c r="R18">
@@ -2734,8 +3107,28 @@
         <f>Inputs!$B$13</f>
         <v>880</v>
       </c>
-    </row>
-    <row r="19" spans="5:19" x14ac:dyDescent="0.2">
+      <c r="AC18">
+        <f t="shared" si="0"/>
+        <v>20263.801643488219</v>
+      </c>
+      <c r="AD18">
+        <f t="shared" si="1"/>
+        <v>1675.3299164504992</v>
+      </c>
+      <c r="AE18">
+        <f>(720-L17)*Inputs!$B$19+(L18-720)*Inputs!$B$20</f>
+        <v>1235.3299164504992</v>
+      </c>
+      <c r="AF18">
+        <f t="shared" si="2"/>
+        <v>2035.4854790319407</v>
+      </c>
+      <c r="AG18">
+        <f>Q18*Inputs!$B$20</f>
+        <v>1155.4854790319407</v>
+      </c>
+    </row>
+    <row r="19" spans="5:33" x14ac:dyDescent="0.2">
       <c r="E19" s="9">
         <v>18</v>
       </c>
@@ -2744,7 +3137,7 @@
         <v>9007.0660478574246</v>
       </c>
       <c r="G19">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>1273.7265118182213</v>
       </c>
       <c r="H19">
@@ -2763,7 +3156,7 @@
         <v>841.87882127848752</v>
       </c>
       <c r="M19">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>66.163918203458365</v>
       </c>
       <c r="O19">
@@ -2774,7 +3167,7 @@
         <v>1012.9676892512279</v>
       </c>
       <c r="Q19">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>68.086991458587363</v>
       </c>
       <c r="R19">
@@ -2785,8 +3178,28 @@
         <f>Inputs!$B$13</f>
         <v>880</v>
       </c>
-    </row>
-    <row r="20" spans="5:19" x14ac:dyDescent="0.2">
+      <c r="AC19">
+        <f t="shared" si="0"/>
+        <v>22991.892245164319</v>
+      </c>
+      <c r="AD19">
+        <f t="shared" si="1"/>
+        <v>1588.6056200120372</v>
+      </c>
+      <c r="AE19">
+        <f>M19*Inputs!$B$20</f>
+        <v>1148.6056200120372</v>
+      </c>
+      <c r="AF19">
+        <f t="shared" si="2"/>
+        <v>2061.9901717210769</v>
+      </c>
+      <c r="AG19">
+        <f>Q19*Inputs!$B$20</f>
+        <v>1181.9901717210766</v>
+      </c>
+    </row>
+    <row r="20" spans="5:33" x14ac:dyDescent="0.2">
       <c r="E20" s="9">
         <v>19</v>
       </c>
@@ -2795,7 +3208,7 @@
         <v>10458.204466678902</v>
       </c>
       <c r="G20">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>1451.1384188214779</v>
       </c>
       <c r="H20">
@@ -2814,7 +3227,7 @@
         <v>910.86611357769698</v>
       </c>
       <c r="M20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>68.987292299209457</v>
       </c>
       <c r="O20">
@@ -2825,7 +3238,7 @@
         <v>1082.6092178872495</v>
       </c>
       <c r="Q20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>69.64152863602169</v>
       </c>
       <c r="R20">
@@ -2836,8 +3249,28 @@
         <f>Inputs!$B$13</f>
         <v>880</v>
       </c>
-    </row>
-    <row r="21" spans="5:19" x14ac:dyDescent="0.2">
+      <c r="AC20">
+        <f t="shared" si="0"/>
+        <v>26071.762950740856</v>
+      </c>
+      <c r="AD20">
+        <f t="shared" si="1"/>
+        <v>1637.6193943142762</v>
+      </c>
+      <c r="AE20">
+        <f>M20*Inputs!$B$20</f>
+        <v>1197.6193943142762</v>
+      </c>
+      <c r="AF20">
+        <f t="shared" si="2"/>
+        <v>2088.9769371213365</v>
+      </c>
+      <c r="AG20">
+        <f>Q20*Inputs!$B$20</f>
+        <v>1208.9769371213365</v>
+      </c>
+    </row>
+    <row r="21" spans="5:33" x14ac:dyDescent="0.2">
       <c r="E21" s="9">
         <v>20</v>
       </c>
@@ -2846,7 +3279,7 @@
         <v>12109.499908786096</v>
       </c>
       <c r="G21">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>1651.2954421071936</v>
       </c>
       <c r="H21">
@@ -2865,7 +3298,7 @@
         <v>982.77659622856766</v>
       </c>
       <c r="M21">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>71.910482650870676</v>
       </c>
       <c r="O21">
@@ -2876,7 +3309,7 @@
         <v>1153.8335085377266</v>
       </c>
       <c r="Q21">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>71.224290650477087</v>
       </c>
       <c r="R21">
@@ -2887,8 +3320,28 @@
         <f>Inputs!$B$13</f>
         <v>880</v>
       </c>
-    </row>
-    <row r="22" spans="5:19" x14ac:dyDescent="0.2">
+      <c r="AC21">
+        <f t="shared" si="0"/>
+        <v>29546.488874980882</v>
+      </c>
+      <c r="AD21">
+        <f t="shared" si="1"/>
+        <v>1688.3659788191148</v>
+      </c>
+      <c r="AE21">
+        <f>M21*Inputs!$B$20</f>
+        <v>1248.3659788191148</v>
+      </c>
+      <c r="AF21">
+        <f t="shared" si="2"/>
+        <v>2116.4536856922823</v>
+      </c>
+      <c r="AG21">
+        <f>Q21*Inputs!$B$20</f>
+        <v>1236.4536856922823</v>
+      </c>
+    </row>
+    <row r="22" spans="5:33" x14ac:dyDescent="0.2">
       <c r="O22">
         <v>21</v>
       </c>
@@ -2897,7 +3350,7 @@
         <v>1226.6692487641703</v>
       </c>
       <c r="Q22">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>72.835740226443704</v>
       </c>
       <c r="R22">
@@ -2908,8 +3361,16 @@
         <f>Inputs!$B$13</f>
         <v>880</v>
       </c>
-    </row>
-    <row r="23" spans="5:19" x14ac:dyDescent="0.2">
+      <c r="AF22">
+        <f t="shared" si="2"/>
+        <v>2144.4284503310628</v>
+      </c>
+      <c r="AG22">
+        <f>Q22*Inputs!$B$20</f>
+        <v>1264.4284503310625</v>
+      </c>
+    </row>
+    <row r="23" spans="5:33" x14ac:dyDescent="0.2">
       <c r="O23">
         <v>22</v>
       </c>
@@ -2918,7 +3379,7 @@
         <v>1301.1455960105666</v>
       </c>
       <c r="Q23">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>74.476347246396244</v>
       </c>
       <c r="R23">
@@ -2929,8 +3390,16 @@
         <f>Inputs!$B$13</f>
         <v>880</v>
       </c>
-    </row>
-    <row r="24" spans="5:19" x14ac:dyDescent="0.2">
+      <c r="AF23">
+        <f t="shared" si="2"/>
+        <v>2172.9093881974386</v>
+      </c>
+      <c r="AG23">
+        <f>Q23*Inputs!$B$20</f>
+        <v>1292.9093881974388</v>
+      </c>
+    </row>
+    <row r="24" spans="5:33" x14ac:dyDescent="0.2">
       <c r="O24">
         <v>23</v>
       </c>
@@ -2939,7 +3408,7 @@
         <v>1377.292184868003</v>
       </c>
       <c r="Q24">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>76.146588857436427</v>
       </c>
       <c r="R24">
@@ -2950,8 +3419,16 @@
         <f>Inputs!$B$13</f>
         <v>880</v>
       </c>
-    </row>
-    <row r="25" spans="5:19" x14ac:dyDescent="0.2">
+      <c r="AF24">
+        <f t="shared" si="2"/>
+        <v>2201.9047825650964</v>
+      </c>
+      <c r="AG24">
+        <f>Q24*Inputs!$B$20</f>
+        <v>1321.9047825650964</v>
+      </c>
+    </row>
+    <row r="25" spans="5:33" x14ac:dyDescent="0.2">
       <c r="O25">
         <v>24</v>
       </c>
@@ -2960,7 +3437,7 @@
         <v>1455.1391344474989</v>
       </c>
       <c r="Q25">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>77.846949579495913</v>
       </c>
       <c r="R25">
@@ -2971,8 +3448,16 @@
         <f>Inputs!$B$13</f>
         <v>880</v>
       </c>
-    </row>
-    <row r="26" spans="5:19" x14ac:dyDescent="0.2">
+      <c r="AF25">
+        <f t="shared" si="2"/>
+        <v>2231.4230447000491</v>
+      </c>
+      <c r="AG25">
+        <f>Q25*Inputs!$B$20</f>
+        <v>1351.4230447000491</v>
+      </c>
+    </row>
+    <row r="26" spans="5:33" x14ac:dyDescent="0.2">
       <c r="O26">
         <v>25</v>
       </c>
@@ -2981,7 +3466,7 @@
         <v>1534.7170558625965</v>
       </c>
       <c r="Q26">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>79.577921415097535</v>
       </c>
       <c r="R26">
@@ -2992,8 +3477,16 @@
         <f>Inputs!$B$13</f>
         <v>880</v>
       </c>
-    </row>
-    <row r="27" spans="5:19" x14ac:dyDescent="0.2">
+      <c r="AF26">
+        <f t="shared" si="2"/>
+        <v>2261.4727157660932</v>
+      </c>
+      <c r="AG26">
+        <f>Q26*Inputs!$B$20</f>
+        <v>1381.4727157660932</v>
+      </c>
+    </row>
+    <row r="27" spans="5:33" x14ac:dyDescent="0.2">
       <c r="O27">
         <v>26</v>
       </c>
@@ -3002,7 +3495,7 @@
         <v>1616.0570598233144</v>
       </c>
       <c r="Q27">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>81.340003960717922</v>
       </c>
       <c r="R27">
@@ -3013,8 +3506,16 @@
         <f>Inputs!$B$13</f>
         <v>880</v>
       </c>
-    </row>
-    <row r="28" spans="5:19" x14ac:dyDescent="0.2">
+      <c r="AF27">
+        <f t="shared" si="2"/>
+        <v>2292.062468758063</v>
+      </c>
+      <c r="AG27">
+        <f>Q27*Inputs!$B$20</f>
+        <v>1412.062468758063</v>
+      </c>
+    </row>
+    <row r="28" spans="5:33" x14ac:dyDescent="0.2">
       <c r="O28">
         <v>27</v>
       </c>
@@ -3023,7 +3524,7 @@
         <v>1699.1907643430709</v>
       </c>
       <c r="Q28">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>83.13370451975652</v>
       </c>
       <c r="R28">
@@ -3034,8 +3535,16 @@
         <f>Inputs!$B$13</f>
         <v>880</v>
       </c>
-    </row>
-    <row r="29" spans="5:19" x14ac:dyDescent="0.2">
+      <c r="AF28">
+        <f t="shared" si="2"/>
+        <v>2323.2011104629732</v>
+      </c>
+      <c r="AG28">
+        <f>Q28*Inputs!$B$20</f>
+        <v>1443.2011104629732</v>
+      </c>
+    </row>
+    <row r="29" spans="5:33" x14ac:dyDescent="0.2">
       <c r="O29">
         <v>28</v>
       </c>
@@ -3044,7 +3553,7 @@
         <v>1784.1503025602246</v>
       </c>
       <c r="Q29">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>84.959538217153749</v>
       </c>
       <c r="R29">
@@ -3055,8 +3564,16 @@
         <f>Inputs!$B$13</f>
         <v>880</v>
       </c>
-    </row>
-    <row r="30" spans="5:19" x14ac:dyDescent="0.2">
+      <c r="AF29">
+        <f t="shared" si="2"/>
+        <v>2354.8975834497887</v>
+      </c>
+      <c r="AG29">
+        <f>Q29*Inputs!$B$20</f>
+        <v>1474.897583449789</v>
+      </c>
+    </row>
+    <row r="30" spans="5:33" x14ac:dyDescent="0.2">
       <c r="O30">
         <v>29</v>
       </c>
@@ -3065,7 +3582,7 @@
         <v>1870.9683306758782</v>
       </c>
       <c r="Q30">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>86.818028115653533</v>
       </c>
       <c r="R30">
@@ -3076,8 +3593,16 @@
         <f>Inputs!$B$13</f>
         <v>880</v>
       </c>
-    </row>
-    <row r="31" spans="5:19" x14ac:dyDescent="0.2">
+      <c r="AF30">
+        <f t="shared" si="2"/>
+        <v>2387.1609680877455</v>
+      </c>
+      <c r="AG30">
+        <f>Q30*Inputs!$B$20</f>
+        <v>1507.1609680877452</v>
+      </c>
+    </row>
+    <row r="31" spans="5:33" x14ac:dyDescent="0.2">
       <c r="O31">
         <v>30</v>
       </c>
@@ -3086,7 +3611,7 @@
         <v>1959.6780360096488</v>
       </c>
       <c r="Q31">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>88.709705333770671</v>
       </c>
       <c r="R31">
@@ -3096,6 +3621,14 @@
       <c r="S31">
         <f>Inputs!$B$13</f>
         <v>880</v>
+      </c>
+      <c r="AF31">
+        <f t="shared" si="2"/>
+        <v>2420.0004845942585</v>
+      </c>
+      <c r="AG31">
+        <f>Q31*Inputs!$B$20</f>
+        <v>1540.0004845942588</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update optimized planting plan and checks
</commit_message>
<xml_diff>
--- a/capabilities/marginal-analysis/model.xlsx
+++ b/capabilities/marginal-analysis/model.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/talaivosamoala/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15AE96D9-0BD2-4F41-A763-E66173CB1049}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF2DB215-D4AB-FE4F-923E-674FD3933A26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="17180" yWindow="940" windowWidth="16880" windowHeight="19360" firstSheet="3" activeTab="9" xr2:uid="{C0270FAA-BF4C-9A43-9A85-05328FDD9A3B}"/>
   </bookViews>
@@ -1246,7 +1246,7 @@
         <v>25</v>
       </c>
       <c r="B2" s="4">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>26</v>
@@ -1268,7 +1268,7 @@
         <v>28</v>
       </c>
       <c r="B4" s="4">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>26</v>
@@ -1306,7 +1306,7 @@
       </c>
       <c r="B2" s="4">
         <f>Beds!B2*Inputs!B11</f>
-        <v>14080</v>
+        <v>8800</v>
       </c>
       <c r="C2" t="s">
         <v>31</v>
@@ -1330,7 +1330,7 @@
       </c>
       <c r="B4" s="4">
         <f>Beds!B4*Inputs!B13</f>
-        <v>24640</v>
+        <v>26400</v>
       </c>
       <c r="C4" t="s">
         <v>34</v>
@@ -1342,7 +1342,7 @@
       </c>
       <c r="B5" s="4">
         <f>B2+B3+B4</f>
-        <v>47520</v>
+        <v>44000</v>
       </c>
       <c r="C5" t="s">
         <v>36</v>
@@ -1380,7 +1380,7 @@
       </c>
       <c r="B2" s="4">
         <f>Beds!B2*Inputs!B5</f>
-        <v>140800</v>
+        <v>88000</v>
       </c>
       <c r="C2" t="s">
         <v>45</v>
@@ -1404,7 +1404,7 @@
       </c>
       <c r="B4" s="4">
         <f>Beds!B4*Inputs!B7</f>
-        <v>75600</v>
+        <v>81000</v>
       </c>
       <c r="C4" t="s">
         <v>42</v>
@@ -1416,7 +1416,7 @@
       </c>
       <c r="B5" s="4">
         <f>B2+B3+B4</f>
-        <v>258280</v>
+        <v>210880</v>
       </c>
       <c r="C5" t="s">
         <v>44</v>
@@ -1454,7 +1454,7 @@
       </c>
       <c r="B2">
         <f>Beds!B2*Inputs!B8*Inputs!B17</f>
-        <v>1440</v>
+        <v>900</v>
       </c>
       <c r="C2" t="s">
         <v>47</v>
@@ -1478,7 +1478,7 @@
       </c>
       <c r="B4">
         <f>Beds!B4*Inputs!B10*Inputs!B17</f>
-        <v>1260</v>
+        <v>1350</v>
       </c>
       <c r="C4" t="s">
         <v>50</v>
@@ -1490,7 +1490,7 @@
       </c>
       <c r="B5">
         <f>B2+B3+B4</f>
-        <v>3299.76</v>
+        <v>2849.76</v>
       </c>
       <c r="C5" t="s">
         <v>53</v>
@@ -1528,7 +1528,7 @@
       </c>
       <c r="B2">
         <f>Beds!B2+Beds!B3+Beds!B4</f>
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="C2" t="s">
         <v>55</v>
@@ -1635,7 +1635,7 @@
       </c>
       <c r="B3" s="6">
         <f>Field_Hours!B5-B2</f>
-        <v>2579.7600000000002</v>
+        <v>2129.7600000000002</v>
       </c>
       <c r="C3" t="s">
         <v>67</v>
@@ -1709,7 +1709,7 @@
       </c>
       <c r="B3" s="6">
         <f>Labor!B3*Inputs!B20</f>
-        <v>44784.633600000001</v>
+        <v>36972.633600000001</v>
       </c>
       <c r="C3" t="s">
         <v>75</v>

</xml_diff>